<commit_message>
Tag CAS ud af årsplanen og resten af materialet
Forkortelsen er væk alle de steder, ungerne kan se den: forløbsnavnene i
årsplanen på siden og i regnearket, de to læringsmål, og lektiearket til uge 39.

Læringsmålene siger nu det samme med ord, de kender: løse ligninger både i
hånden og med et regneprogram, og bruge et regneprogram og vurdere, om svaret er
rimeligt. På uge 39-arket står der GeoGebra, som er det program klassen faktisk
bruger.

Filen er omdøbt til kommende/lektier-uge39-ligninger-fortsat.html, så navnet
heller ikke bærer forkortelsen rundt.

Både siden og regnearket er rettet, og claude/tjek.py bekræfter, at de 23 forløb
stadig står ens begge steder.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VgEVctXq3tNeZxt6iAFBPu
</commit_message>
<xml_diff>
--- a/aarsplan-matematik-2026-27.xlsx
+++ b/aarsplan-matematik-2026-27.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Årsplan" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Overblik" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Projektopgave" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Årsplan" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overblik" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projektopgave" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Årsplan'!$4:$4</definedName>
@@ -701,6 +701,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="24" customHeight="1" s="28">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -935,13 +936,13 @@
       </c>
       <c r="D12" s="37" t="inlineStr">
         <is>
-          <t>Ligninger og CAS</t>
+          <t>Ligninger</t>
         </is>
       </c>
       <c r="E12" s="38" t="inlineStr">
         <is>
           <t>Opstille ligninger til at løse problemer fra virkeligheden
-Løse ligninger med og uden brug af CAS
+Løse ligninger både i hånden og med et regneprogram
 Vælge hensigtsmæssige strategier til løsning af ligninger</t>
         </is>
       </c>
@@ -968,13 +969,13 @@
       </c>
       <c r="D13" s="37" t="inlineStr">
         <is>
-          <t>Ligninger og CAS (fortsat)</t>
+          <t>Ligninger (fortsat)</t>
         </is>
       </c>
       <c r="E13" s="38" t="inlineStr">
         <is>
           <t>Løse ligninger med parenteser, brøker og x på begge sider
-Bruge CAS-værktøj og vurdere resultatet</t>
+Bruge et regneprogram og vurdere, om svaret er rimeligt</t>
         </is>
       </c>
       <c r="F13" s="38" t="n"/>

</xml_diff>